<commit_message>
Make 102LA a single-head dwarf without shifting C4 packed IDs.
Keep IH434 on the mast, leave IH435 as a spare port, and align CATS, USS, tables, and wiring docs before the rename.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/wiring/signals_asbuilt_abs_v2.xlsx
+++ b/docs/wiring/signals_asbuilt_abs_v2.xlsx
@@ -1147,7 +1147,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O24"/>
+  <dimension ref="A1:O25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -1327,7 +1327,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -1352,64 +1352,52 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>434 435</t>
+          <t>434</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>C4-OU2-3 C4-OU2-4</t>
+          <t>C4-OU2-3</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>track/signalhead/IH434 track/signalhead/IH435</t>
+          <t>track/signalhead/IH434</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH434)(IH435)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH434)</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '102LA'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '102LA' (1-head; was Top of 2-head)</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Brick</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>101RA</t>
-        </is>
-      </c>
+          <t>West - Lower</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr"/>
       <c r="C4" t="n">
         <v>1</v>
       </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>left</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>(4,3) LEFT</t>
-        </is>
-      </c>
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
@@ -1423,24 +1411,20 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>436</t>
+          <t>435</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>C4-OU2-5</t>
+          <t>C4-OU2-4</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>track/signalhead/IH436</t>
-        </is>
-      </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
-        </is>
-      </c>
+          <t>track/signalhead/IH435</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr">
         <is>
           <t>single</t>
@@ -1453,7 +1437,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '101RA'</t>
+          <t>LCOS Signal 3 UID 35; spare (was 102LA Bottom); packed slot held so 101RA stays IH436</t>
         </is>
       </c>
     </row>
@@ -1465,7 +1449,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>101RB</t>
+          <t>101RA</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1478,7 +1462,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(4,4) LEFT</t>
+          <t>(4,3) LEFT</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -1494,22 +1478,22 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>437</t>
+          <t>436</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>C4-OU2-6</t>
+          <t>C4-OU2-5</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>track/signalhead/IH437</t>
+          <t>track/signalhead/IH436</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH436)</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
@@ -1524,7 +1508,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '101RB'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '101RA'</t>
         </is>
       </c>
     </row>
@@ -1536,20 +1520,20 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>100L</t>
+          <t>101RB</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(8,3) RIGHT</t>
+          <t>(4,4) LEFT</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -1565,49 +1549,49 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>438 439</t>
+          <t>437</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>C4-OU3-1 C4-OU3-2</t>
+          <t>C4-OU2-6</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>track/signalhead/IH438 track/signalhead/IH439</t>
+          <t>track/signalhead/IH437</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH438)(IH439)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH437)</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>LCOS Signal 6 UID 38; Digicon mast '100L'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '101RB'</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>West Yard</t>
+          <t>Brick</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>117RA</t>
+          <t>100L</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1615,43 +1599,43 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>(12,7) LEFT</t>
+          <t>(8,3) RIGHT</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>C1</t>
+          <t>C4</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1332 1333</t>
+          <t>438 439</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>C1-OU2-1 C1-OU2-2</t>
+          <t>C4-OU3-1 C4-OU3-2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1332 track/signalhead/IH1333</t>
+          <t>track/signalhead/IH438 track/signalhead/IH439</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1332)(IH1333)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH438)(IH439)</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
@@ -1666,7 +1650,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '117RA'</t>
+          <t>LCOS Signal 6 UID 38; Digicon mast '100L'</t>
         </is>
       </c>
     </row>
@@ -1678,20 +1662,20 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>117LB</t>
+          <t>117RA</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(14,7) RIGHT</t>
+          <t>(12,7) LEFT</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -1707,37 +1691,37 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1334</t>
+          <t>1332 1333</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>C1-OU2-3</t>
+          <t>C1-OU2-1 C1-OU2-2</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1334</t>
+          <t>track/signalhead/IH1332 track/signalhead/IH1333</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1332)(IH1333)</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low</t>
+          <t>hart-aar SL-2-digicon</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '117LB'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '117RA'</t>
         </is>
       </c>
     </row>
@@ -1749,20 +1733,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>117RB</t>
+          <t>117LB</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(12,8) LEFT</t>
+          <t>(14,7) RIGHT</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -1778,37 +1762,37 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1335 1336</t>
+          <t>1334</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>C1-OU2-4 C1-OU2-5</t>
+          <t>C1-OU2-3</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1335 track/signalhead/IH1336</t>
+          <t>track/signalhead/IH1334</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1335)(IH1336)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1334)</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '117RB'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '117LB'</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1804,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>117LA</t>
+          <t>117RB</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1828,12 +1812,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(14,8) RIGHT</t>
+          <t>(12,8) LEFT</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1849,22 +1833,22 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1337 1338</t>
+          <t>1335 1336</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>C1-OU2-6 C1-OU3-1</t>
+          <t>C1-OU2-4 C1-OU2-5</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1337 track/signalhead/IH1338</t>
+          <t>track/signalhead/IH1335 track/signalhead/IH1336</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1337)(IH1338)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1335)(IH1336)</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
@@ -1879,19 +1863,19 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '117LA'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '117RB'</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>East End</t>
+          <t>West Yard</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>111RA</t>
+          <t>117LA</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1899,43 +1883,43 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(28,6) LEFT</t>
+          <t>(14,8) RIGHT</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>13</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>C7</t>
+          <t>C1</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1232 1233</t>
+          <t>1337 1338</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>C7-OU2-1 C7-OU2-2</t>
+          <t>C1-OU2-6 C1-OU3-1</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1232 track/signalhead/IH1233</t>
+          <t>track/signalhead/IH1337 track/signalhead/IH1338</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1232)(IH1233)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1337)(IH1338)</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
@@ -1950,7 +1934,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '111RA'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '117LA'</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1946,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>111L</t>
+          <t>111RA</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1970,12 +1954,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>(30,6) RIGHT</t>
+          <t>(28,6) LEFT</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1991,22 +1975,22 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1234 1235</t>
+          <t>1232 1233</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>C7-OU2-3 C7-OU2-4</t>
+          <t>C7-OU2-1 C7-OU2-2</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1234 track/signalhead/IH1235</t>
+          <t>track/signalhead/IH1232 track/signalhead/IH1233</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1234)(IH1235)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1232)(IH1233)</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
@@ -2021,7 +2005,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '111L'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '111RA'</t>
         </is>
       </c>
     </row>
@@ -2033,20 +2017,20 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>111RB</t>
+          <t>111L</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>(28,7) LEFT</t>
+          <t>(30,6) RIGHT</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -2062,37 +2046,37 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1236</t>
+          <t>1234 1235</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>C7-OU2-5</t>
+          <t>C7-OU2-3 C7-OU2-4</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1236</t>
+          <t>track/signalhead/IH1234 track/signalhead/IH1235</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1236)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1234)(IH1235)</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low</t>
+          <t>hart-aar SL-2-digicon</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>LCOS Signal 4 UID 36; Digicon mast '111RB'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '111L'</t>
         </is>
       </c>
     </row>
@@ -2104,20 +2088,20 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>112L</t>
+          <t>111RB</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>(34,7) RIGHT</t>
+          <t>(28,7) LEFT</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -2133,37 +2117,37 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1237 1238</t>
+          <t>1236</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>C7-OU2-6 C7-OU3-1</t>
+          <t>C7-OU2-5</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1237 track/signalhead/IH1238</t>
+          <t>track/signalhead/IH1236</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1237)(IH1238)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1236)</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '112L'</t>
+          <t>LCOS Signal 4 UID 36; Digicon mast '111RB'</t>
         </is>
       </c>
     </row>
@@ -2175,20 +2159,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>110R</t>
+          <t>112L</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>bottom</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>(31,7) BOTTOM</t>
+          <t>(34,7) RIGHT</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -2204,37 +2188,37 @@
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1239</t>
+          <t>1237 1238</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>C7-OU3-2</t>
+          <t>C7-OU2-6 C7-OU3-1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1239</t>
+          <t>track/signalhead/IH1237 track/signalhead/IH1238</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH1239)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1237)(IH1238)</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low</t>
+          <t>hart-aar SL-2-digicon</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '110R'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '112L'</t>
         </is>
       </c>
     </row>
@@ -2246,20 +2230,20 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>112R</t>
+          <t>110R</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>bottom</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>(33,8) LEFT</t>
+          <t>(31,7) BOTTOM</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -2275,49 +2259,49 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1240 1241</t>
+          <t>1239</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>C7-OU3-3 C7-OU3-4</t>
+          <t>C7-OU3-2</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>track/signalhead/IH1240 track/signalhead/IH1241</t>
+          <t>track/signalhead/IH1239</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1240)(IH1241)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH1239)</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>LCOS Signal 8 UID 40; Digicon mast '112R'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '110R'</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Princess</t>
+          <t>East End</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>115LB</t>
+          <t>112R</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -2325,43 +2309,43 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(43,5) RIGHT</t>
+          <t>(33,8) LEFT</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>12</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>C7</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>132 133</t>
+          <t>1240 1241</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>D1-OU2-1 D1-OU2-2</t>
+          <t>C7-OU3-3 C7-OU3-4</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>track/signalhead/IH132 track/signalhead/IH133</t>
+          <t>track/signalhead/IH1240 track/signalhead/IH1241</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH132)(IH133)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH1240)(IH1241)</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
@@ -2376,7 +2360,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>LCOS Signal 0 UID 32; Digicon mast '115LB'</t>
+          <t>LCOS Signal 8 UID 40; Digicon mast '112R'</t>
         </is>
       </c>
     </row>
@@ -2388,20 +2372,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>114R</t>
+          <t>115LB</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>top</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(45,7) TOP</t>
+          <t>(43,5) RIGHT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -2417,37 +2401,37 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>134</t>
+          <t>132 133</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>D1-OU2-3</t>
+          <t>D1-OU2-1 D1-OU2-2</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>track/signalhead/IH134</t>
+          <t>track/signalhead/IH132 track/signalhead/IH133</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH134)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH132)(IH133)</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low</t>
+          <t>hart-aar SL-2-digicon</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>LCOS Signal 2 UID 34; Digicon mast '114R'</t>
+          <t>LCOS Signal 0 UID 32; Digicon mast '115LB'</t>
         </is>
       </c>
     </row>
@@ -2459,20 +2443,20 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>113RA</t>
+          <t>114R</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>top</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>(37,6) LEFT</t>
+          <t>(45,7) TOP</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -2488,37 +2472,37 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>135 136</t>
+          <t>134</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>D1-OU2-4 D1-OU2-5</t>
+          <t>D1-OU2-3</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>track/signalhead/IH135 track/signalhead/IH136</t>
+          <t>track/signalhead/IH134</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH135)(IH136)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH134)</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>double</t>
+          <t>single</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>hart-aar SL-2-digicon</t>
+          <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>LCOS Signal 3 UID 35; Digicon mast '113RA'</t>
+          <t>LCOS Signal 2 UID 34; Digicon mast '114R'</t>
         </is>
       </c>
     </row>
@@ -2530,7 +2514,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>113RB</t>
+          <t>113RA</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -2543,7 +2527,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>(37,7) LEFT</t>
+          <t>(37,6) LEFT</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -2559,22 +2543,22 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>137 138</t>
+          <t>135 136</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>D1-OU2-6 D1-OU2-7</t>
+          <t>D1-OU2-4 D1-OU2-5</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>track/signalhead/IH137 track/signalhead/IH138</t>
+          <t>track/signalhead/IH135 track/signalhead/IH136</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH137)(IH138)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH135)(IH136)</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
@@ -2589,7 +2573,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>LCOS Signal 5 UID 37; Digicon mast '113RB'</t>
+          <t>LCOS Signal 3 UID 35; Digicon mast '113RA'</t>
         </is>
       </c>
     </row>
@@ -2601,7 +2585,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>114LB</t>
+          <t>113RB</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -2609,12 +2593,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>right</t>
+          <t>left</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>(43,8) RIGHT</t>
+          <t>(37,7) LEFT</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -2630,22 +2614,22 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>139 140</t>
+          <t>137 138</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>D1-OU2-8 D1-OU3-1</t>
+          <t>D1-OU2-6 D1-OU2-7</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>track/signalhead/IH139 track/signalhead/IH140</t>
+          <t>track/signalhead/IH137 track/signalhead/IH138</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH139)(IH140)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH137)(IH138)</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
@@ -2660,7 +2644,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>LCOS Signal 7 UID 39; Digicon mast '114LB'</t>
+          <t>LCOS Signal 5 UID 37; Digicon mast '113RB'</t>
         </is>
       </c>
     </row>
@@ -2672,20 +2656,20 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>115R</t>
+          <t>114LB</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>bottom</t>
+          <t>right</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>(45,6) BOTTOM</t>
+          <t>(43,8) RIGHT</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -2701,37 +2685,37 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>141</t>
+          <t>139 140</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>D1-OU3-2</t>
+          <t>D1-OU2-8 D1-OU3-1</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>track/signalhead/IH141</t>
+          <t>track/signalhead/IH139 track/signalhead/IH140</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH141)</t>
+          <t>IF$shsm:AAR-1946:SL-2-high-abs(IH139)(IH140)</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>single</t>
+          <t>double</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>AAR-1946 SL-1-low</t>
+          <t>hart-aar SL-2-digicon</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>LCOS Signal 9 UID 41; Digicon mast '115R'</t>
+          <t>LCOS Signal 7 UID 39; Digicon mast '114LB'</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2727,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>115LA</t>
+          <t>115R</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -2751,12 +2735,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>left</t>
+          <t>bottom</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(43,6) RIGHT</t>
+          <t>(45,6) BOTTOM</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -2772,22 +2756,22 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>142</t>
+          <t>141</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>D1-OU3-3</t>
+          <t>D1-OU3-2</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>track/signalhead/IH142</t>
+          <t>track/signalhead/IH141</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH141)</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
@@ -2802,7 +2786,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>LCOS Signal 10 UID 42; Digicon mast '115LA'</t>
+          <t>LCOS Signal 9 UID 41; Digicon mast '115R'</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2798,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>114LA</t>
+          <t>115LA</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -2827,7 +2811,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>(43,7) RIGHT</t>
+          <t>(43,6) RIGHT</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -2843,35 +2827,106 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
+          <t>142</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>D1-OU3-3</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>track/signalhead/IH142</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>IF$shsm:AAR-1946:SL-1-low(IH142)</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>single</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>AAR-1946 SL-1-low</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>LCOS Signal 10 UID 42; Digicon mast '115LA'</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Princess</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>114LA</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>left</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>(43,7) RIGHT</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
           <t>143</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J25" t="inlineStr">
         <is>
           <t>D1-OU3-4</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
+      <c r="K25" t="inlineStr">
         <is>
           <t>track/signalhead/IH143</t>
         </is>
       </c>
-      <c r="L24" t="inlineStr">
+      <c r="L25" t="inlineStr">
         <is>
           <t>IF$shsm:AAR-1946:SL-1-low(IH143)</t>
         </is>
       </c>
-      <c r="M24" t="inlineStr">
+      <c r="M25" t="inlineStr">
         <is>
           <t>single</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr">
+      <c r="N25" t="inlineStr">
         <is>
           <t>AAR-1946 SL-1-low</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
+      <c r="O25" t="inlineStr">
         <is>
           <t>LCOS Signal 11 UID 43; Digicon mast '114LA'</t>
         </is>
@@ -19185,7 +19240,7 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>EH-1</t>
+          <t>EH-3</t>
         </is>
       </c>
       <c r="C40" s="3" t="inlineStr">
@@ -19200,7 +19255,7 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
-          <t>EH-1</t>
+          <t>EH-3</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -19249,7 +19304,7 @@
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>EH-3</t>
+          <t>EH-1</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
@@ -19264,7 +19319,7 @@
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>EH-3</t>
+          <t>EH-1</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">

</xml_diff>